<commit_message>
atualização do codigo base
</commit_message>
<xml_diff>
--- a/9 -  MB25/MB25 ATUALIZADA.xlsx
+++ b/9 -  MB25/MB25 ATUALIZADA.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20369" uniqueCount="2217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20381" uniqueCount="2218">
   <si>
     <t>Reserva</t>
   </si>
@@ -6662,6 +6662,9 @@
   </si>
   <si>
     <t>60001704</t>
+  </si>
+  <si>
+    <t>325322</t>
   </si>
 </sst>
 </file>
@@ -6783,7 +6786,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1"/>
   </sheetPr>
-  <dimension ref="A1:Q1697"/>
+  <dimension ref="A1:Q1698"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" bestFit="1" width="8" customWidth="1"/>
@@ -96746,6 +96749,59 @@
         <v>2216</v>
       </c>
     </row>
+    <row r="1698" outlineLevel="0" collapsed="0" hidden="0">
+      <c r="A1698" s="2" t="s">
+        <v>2217</v>
+      </c>
+      <c r="B1698" s="2" t="s">
+        <v>1333</v>
+      </c>
+      <c r="C1698" s="5">
+        <v>2.000</v>
+      </c>
+      <c r="D1698" s="4">
+        <v>46227</v>
+      </c>
+      <c r="E1698" s="4">
+        <v>46227</v>
+      </c>
+      <c r="F1698" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1698" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H1698" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="I1698" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1698" s="3">
+        <v>0</v>
+      </c>
+      <c r="K1698" s="5">
+        <v>2.000</v>
+      </c>
+      <c r="L1698" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M1698" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N1698" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="O1698" s="2" t="s">
+        <v>2170</v>
+      </c>
+      <c r="P1698" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q1698" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>